<commit_message>
fixed Kurile 1969 event reference
</commit_message>
<xml_diff>
--- a/data_compilation.xlsx
+++ b/data_compilation.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adminalba/Documents/Paleoseismology compilation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/albamarrodriguezpadilla/Downloads/paleoseismology_subduction-main/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4582212C-32D9-4845-8D27-2109524BBDDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B5BA4C4-20FF-B448-AEFB-446668F63447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{0C72CEA8-103F-664E-BFC3-8082C479B46F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="148">
   <si>
     <t>Year</t>
   </si>
@@ -330,9 +330,6 @@
   </si>
   <si>
     <t>Hokkaido Segment</t>
-  </si>
-  <si>
-    <t>Nanayama et al., 2007, Satake et al. 2008</t>
   </si>
   <si>
     <t>Nanayama et al., 2007, Satake et al. 2009</t>
@@ -558,9 +555,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -598,7 +595,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -704,7 +701,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -846,7 +843,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -857,8 +854,9 @@
   <dimension ref="A1:I209"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="5" max="5" width="7.6640625" customWidth="1"/>
-    <col min="6" max="7" width="19.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.33203125" customWidth="1"/>
+    <col min="6" max="6" width="30.33203125" customWidth="1"/>
+    <col min="7" max="7" width="25.1640625" customWidth="1"/>
     <col min="8" max="8" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -867,13 +865,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C1" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1" t="s">
         <v>137</v>
-      </c>
-      <c r="C1" t="s">
-        <v>136</v>
-      </c>
-      <c r="D1" t="s">
-        <v>138</v>
       </c>
       <c r="E1" t="s">
         <v>1</v>
@@ -925,7 +923,7 @@
         <v>2.5</v>
       </c>
       <c r="D3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F3" t="s">
         <v>6</v>
@@ -951,7 +949,7 @@
         <v>3.5</v>
       </c>
       <c r="D4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F4" t="s">
         <v>7</v>
@@ -977,7 +975,7 @@
         <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F5" t="s">
         <v>8</v>
@@ -1003,7 +1001,7 @@
         <v>6.6</v>
       </c>
       <c r="D6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F6" t="s">
         <v>9</v>
@@ -1029,7 +1027,7 @@
         <v>8.6999999999999993</v>
       </c>
       <c r="D7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F7" t="s">
         <v>10</v>
@@ -1055,7 +1053,7 @@
         <v>11.4</v>
       </c>
       <c r="D8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F8" t="s">
         <v>11</v>
@@ -1081,7 +1079,7 @@
         <v>2.5</v>
       </c>
       <c r="D9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E9" t="s">
         <v>12</v>
@@ -1110,7 +1108,7 @@
         <v>2.4</v>
       </c>
       <c r="D10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F10" t="s">
         <v>15</v>
@@ -1136,7 +1134,7 @@
         <v>2.5</v>
       </c>
       <c r="D11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F11" t="s">
         <v>15</v>
@@ -1162,7 +1160,7 @@
         <v>0</v>
       </c>
       <c r="D12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F12" t="s">
         <v>20</v>
@@ -1188,7 +1186,7 @@
         <v>17</v>
       </c>
       <c r="D13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F13" t="s">
         <v>20</v>
@@ -1214,7 +1212,7 @@
         <v>0.8</v>
       </c>
       <c r="D14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F14" t="s">
         <v>21</v>
@@ -1240,7 +1238,7 @@
         <v>0</v>
       </c>
       <c r="D15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F15" t="s">
         <v>21</v>
@@ -1266,7 +1264,7 @@
         <v>0.5</v>
       </c>
       <c r="D16" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E16" t="s">
         <v>18</v>
@@ -1295,7 +1293,7 @@
         <v>0</v>
       </c>
       <c r="D17" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F17" t="s">
         <v>23</v>
@@ -1321,7 +1319,7 @@
         <v>1.7</v>
       </c>
       <c r="D18" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E18" t="s">
         <v>19</v>
@@ -1350,7 +1348,7 @@
         <v>-0.5</v>
       </c>
       <c r="D19" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F19" t="s">
         <v>26</v>
@@ -1376,7 +1374,7 @@
         <v>5</v>
       </c>
       <c r="D20" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F20" t="s">
         <v>27</v>
@@ -1402,7 +1400,7 @@
         <v>-3.6</v>
       </c>
       <c r="D21" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E21" t="s">
         <v>18</v>
@@ -1431,7 +1429,7 @@
         <v>-4.5</v>
       </c>
       <c r="D22" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F22" t="s">
         <v>30</v>
@@ -1457,7 +1455,7 @@
         <v>-3.5</v>
       </c>
       <c r="D23" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F23" t="s">
         <v>30</v>
@@ -1483,7 +1481,7 @@
         <v>-3.5</v>
       </c>
       <c r="D24" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F24" t="s">
         <v>31</v>
@@ -1509,7 +1507,7 @@
         <v>-3.7</v>
       </c>
       <c r="D25" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F25" t="s">
         <v>31</v>
@@ -1535,7 +1533,7 @@
         <v>-4</v>
       </c>
       <c r="D26" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E26" t="s">
         <v>19</v>
@@ -1564,7 +1562,7 @@
         <v>-2.5</v>
       </c>
       <c r="D27" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F27" t="s">
         <v>31</v>
@@ -1590,7 +1588,7 @@
         <v>-4.5</v>
       </c>
       <c r="D28" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F28" t="s">
         <v>31</v>
@@ -1616,7 +1614,7 @@
         <v>-3.4</v>
       </c>
       <c r="D29" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F29" t="s">
         <v>32</v>
@@ -1642,7 +1640,7 @@
         <v>-4.5</v>
       </c>
       <c r="D30" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F30" t="s">
         <v>32</v>
@@ -1668,7 +1666,7 @@
         <v>-4.5</v>
       </c>
       <c r="D31" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F31" t="s">
         <v>33</v>
@@ -1694,7 +1692,7 @@
         <v>-2.8</v>
       </c>
       <c r="D32" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E32" t="s">
         <v>19</v>
@@ -1723,7 +1721,7 @@
         <v>-2</v>
       </c>
       <c r="D33" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E33" t="s">
         <v>19</v>
@@ -1752,7 +1750,7 @@
         <v>-2.7</v>
       </c>
       <c r="D34" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F34" t="s">
         <v>36</v>
@@ -1778,7 +1776,7 @@
         <v>-4</v>
       </c>
       <c r="D35" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E35" t="s">
         <v>18</v>
@@ -1807,7 +1805,7 @@
         <v>-5.7</v>
       </c>
       <c r="D36" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F36" t="s">
         <v>39</v>
@@ -1833,7 +1831,7 @@
         <v>-0.5</v>
       </c>
       <c r="D37" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F37" t="s">
         <v>42</v>
@@ -1859,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="D38" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F38" t="s">
         <v>44</v>
@@ -1885,7 +1883,7 @@
         <v>0</v>
       </c>
       <c r="D39" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F39" t="s">
         <v>42</v>
@@ -1911,7 +1909,7 @@
         <v>-0.5</v>
       </c>
       <c r="D40" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F40" t="s">
         <v>42</v>
@@ -1937,7 +1935,7 @@
         <v>1.2</v>
       </c>
       <c r="D41" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F41" t="s">
         <v>42</v>
@@ -1963,7 +1961,7 @@
         <v>1.7</v>
       </c>
       <c r="D42" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F42" t="s">
         <v>42</v>
@@ -1989,7 +1987,7 @@
         <v>-0.6</v>
       </c>
       <c r="D43" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F43" t="s">
         <v>42</v>
@@ -2015,7 +2013,7 @@
         <v>-0.5</v>
       </c>
       <c r="D44" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F44" t="s">
         <v>46</v>
@@ -2041,7 +2039,7 @@
         <v>-8.5</v>
       </c>
       <c r="D45" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F45" t="s">
         <v>58</v>
@@ -2067,7 +2065,7 @@
         <v>-4.5</v>
       </c>
       <c r="D46" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F46" t="s">
         <v>59</v>
@@ -2093,7 +2091,7 @@
         <v>-5</v>
       </c>
       <c r="D47" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F47" t="s">
         <v>59</v>
@@ -2119,7 +2117,7 @@
         <v>-7.5</v>
       </c>
       <c r="D48" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E48" t="s">
         <v>18</v>
@@ -2148,7 +2146,7 @@
         <v>-10.199999999999999</v>
       </c>
       <c r="D49" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E49" t="s">
         <v>18</v>
@@ -2177,7 +2175,7 @@
         <v>-13.7</v>
       </c>
       <c r="D50" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F50" t="s">
         <v>61</v>
@@ -2203,7 +2201,7 @@
         <v>-14.8</v>
       </c>
       <c r="D51" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F51" t="s">
         <v>61</v>
@@ -2229,7 +2227,7 @@
         <v>-11.5</v>
       </c>
       <c r="D52" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F52" t="s">
         <v>61</v>
@@ -2255,7 +2253,7 @@
         <v>-15.2</v>
       </c>
       <c r="D53" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F53" t="s">
         <v>61</v>
@@ -2281,7 +2279,7 @@
         <v>-13.5</v>
       </c>
       <c r="D54" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F54" t="s">
         <v>61</v>
@@ -2307,7 +2305,7 @@
         <v>-11.5</v>
       </c>
       <c r="D55" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F55" t="s">
         <v>60</v>
@@ -2333,7 +2331,7 @@
         <v>-11.2</v>
       </c>
       <c r="D56" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F56" t="s">
         <v>60</v>
@@ -2359,7 +2357,7 @@
         <v>-13.5</v>
       </c>
       <c r="D57" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F57" t="s">
         <v>60</v>
@@ -2385,7 +2383,7 @@
         <v>-14</v>
       </c>
       <c r="D58" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F58" t="s">
         <v>60</v>
@@ -2411,7 +2409,7 @@
         <v>-17</v>
       </c>
       <c r="D59" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F59" t="s">
         <v>61</v>
@@ -2437,7 +2435,7 @@
         <v>-18.2</v>
       </c>
       <c r="D60" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F60" t="s">
         <v>61</v>
@@ -2463,7 +2461,7 @@
         <v>-17.5</v>
       </c>
       <c r="D61" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F61" t="s">
         <v>61</v>
@@ -2489,7 +2487,7 @@
         <v>-18</v>
       </c>
       <c r="D62" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F62" t="s">
         <v>61</v>
@@ -2515,7 +2513,7 @@
         <v>-18</v>
       </c>
       <c r="D63" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F63" t="s">
         <v>61</v>
@@ -2541,7 +2539,7 @@
         <v>-18.5</v>
       </c>
       <c r="D64" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F64" t="s">
         <v>61</v>
@@ -2567,7 +2565,7 @@
         <v>-15.8</v>
       </c>
       <c r="D65" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F65" t="s">
         <v>60</v>
@@ -2593,7 +2591,7 @@
         <v>-15.5</v>
       </c>
       <c r="D66" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F66" t="s">
         <v>60</v>
@@ -2619,7 +2617,7 @@
         <v>-17.2</v>
       </c>
       <c r="D67" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F67" t="s">
         <v>60</v>
@@ -2645,7 +2643,7 @@
         <v>-18</v>
       </c>
       <c r="D68" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F68" t="s">
         <v>60</v>
@@ -2671,7 +2669,7 @@
         <v>-20</v>
       </c>
       <c r="D69" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F69" t="s">
         <v>67</v>
@@ -2697,7 +2695,7 @@
         <v>-19</v>
       </c>
       <c r="D70" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F70" t="s">
         <v>67</v>
@@ -2723,7 +2721,7 @@
         <v>-21.5</v>
       </c>
       <c r="D71" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F71" t="s">
         <v>67</v>
@@ -2749,7 +2747,7 @@
         <v>-19.399999999999999</v>
       </c>
       <c r="D72" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F72" t="s">
         <v>68</v>
@@ -2775,7 +2773,7 @@
         <v>-22.5</v>
       </c>
       <c r="D73" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F73" t="s">
         <v>67</v>
@@ -2801,7 +2799,7 @@
         <v>-20</v>
       </c>
       <c r="D74" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F74" t="s">
         <v>67</v>
@@ -2827,7 +2825,7 @@
         <v>-20.7</v>
       </c>
       <c r="D75" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F75" t="s">
         <v>67</v>
@@ -2853,7 +2851,7 @@
         <v>-23</v>
       </c>
       <c r="D76" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F76" t="s">
         <v>67</v>
@@ -2879,7 +2877,7 @@
         <v>-20.5</v>
       </c>
       <c r="D77" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F77" t="s">
         <v>67</v>
@@ -2905,7 +2903,7 @@
         <v>-23.2</v>
       </c>
       <c r="D78" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F78" t="s">
         <v>60</v>
@@ -2931,7 +2929,7 @@
         <v>-20.3</v>
       </c>
       <c r="D79" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F79" t="s">
         <v>69</v>
@@ -2957,7 +2955,7 @@
         <v>-20.7</v>
       </c>
       <c r="D80" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F80" t="s">
         <v>69</v>
@@ -2983,7 +2981,7 @@
         <v>-25</v>
       </c>
       <c r="D81" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F81" t="s">
         <v>60</v>
@@ -3009,7 +3007,7 @@
         <v>-28.5</v>
       </c>
       <c r="D82" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E82" t="s">
         <v>73</v>
@@ -3038,7 +3036,7 @@
         <v>-30</v>
       </c>
       <c r="D83" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E83" t="s">
         <v>74</v>
@@ -3067,7 +3065,7 @@
         <v>-26.5</v>
       </c>
       <c r="D84" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F84" t="s">
         <v>72</v>
@@ -3093,7 +3091,7 @@
         <v>-30.2</v>
       </c>
       <c r="D85" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F85" t="s">
         <v>72</v>
@@ -3119,7 +3117,7 @@
         <v>-34</v>
       </c>
       <c r="D86" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F86" t="s">
         <v>72</v>
@@ -3145,7 +3143,7 @@
         <v>-35</v>
       </c>
       <c r="D87" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F87" t="s">
         <v>72</v>
@@ -3171,7 +3169,7 @@
         <v>-36</v>
       </c>
       <c r="D88" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F88" t="s">
         <v>72</v>
@@ -3197,7 +3195,7 @@
         <v>-33.700000000000003</v>
       </c>
       <c r="D89" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F89" t="s">
         <v>72</v>
@@ -3223,7 +3221,7 @@
         <v>-33.700000000000003</v>
       </c>
       <c r="D90" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F90" t="s">
         <v>72</v>
@@ -3249,7 +3247,7 @@
         <v>-33</v>
       </c>
       <c r="D91" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F91" t="s">
         <v>72</v>
@@ -3275,7 +3273,7 @@
         <v>-32</v>
       </c>
       <c r="D92" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F92" t="s">
         <v>72</v>
@@ -3301,7 +3299,7 @@
         <v>-35</v>
       </c>
       <c r="D93" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F93" t="s">
         <v>72</v>
@@ -3327,7 +3325,7 @@
         <v>-32</v>
       </c>
       <c r="D94" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F94" t="s">
         <v>72</v>
@@ -3353,7 +3351,7 @@
         <v>-33</v>
       </c>
       <c r="D95" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F95" t="s">
         <v>72</v>
@@ -3379,7 +3377,7 @@
         <v>-34.5</v>
       </c>
       <c r="D96" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F96" t="s">
         <v>72</v>
@@ -3405,7 +3403,7 @@
         <v>-32</v>
       </c>
       <c r="D97" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F97" t="s">
         <v>76</v>
@@ -3431,7 +3429,7 @@
         <v>-38</v>
       </c>
       <c r="D98" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F98" t="s">
         <v>78</v>
@@ -3457,7 +3455,7 @@
         <v>-38.5</v>
       </c>
       <c r="D99" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F99" t="s">
         <v>78</v>
@@ -3483,7 +3481,7 @@
         <v>-39</v>
       </c>
       <c r="D100" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F100" t="s">
         <v>78</v>
@@ -3509,7 +3507,7 @@
         <v>-38.5</v>
       </c>
       <c r="D101" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F101" t="s">
         <v>78</v>
@@ -3535,7 +3533,7 @@
         <v>-36</v>
       </c>
       <c r="D102" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F102" t="s">
         <v>72</v>
@@ -3561,7 +3559,7 @@
         <v>-38</v>
       </c>
       <c r="D103" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F103" t="s">
         <v>78</v>
@@ -3587,7 +3585,7 @@
         <v>-38.5</v>
       </c>
       <c r="D104" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F104" t="s">
         <v>79</v>
@@ -3613,7 +3611,7 @@
         <v>-46</v>
       </c>
       <c r="D105" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E105" t="s">
         <v>12</v>
@@ -3642,7 +3640,7 @@
         <v>-46</v>
       </c>
       <c r="D106" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E106" t="s">
         <v>19</v>
@@ -3671,7 +3669,7 @@
         <v>-46</v>
       </c>
       <c r="D107" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E107" t="s">
         <v>12</v>
@@ -3700,7 +3698,7 @@
         <v>-46</v>
       </c>
       <c r="D108" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E108" t="s">
         <v>12</v>
@@ -3729,7 +3727,7 @@
         <v>-43.8</v>
       </c>
       <c r="D109" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F109" t="s">
         <v>81</v>
@@ -3755,7 +3753,7 @@
         <v>138.6</v>
       </c>
       <c r="D110" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F110" t="s">
         <v>85</v>
@@ -3781,7 +3779,7 @@
         <v>138.6</v>
       </c>
       <c r="D111" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F111" t="s">
         <v>85</v>
@@ -3807,7 +3805,7 @@
         <v>138.30000000000001</v>
       </c>
       <c r="D112" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F112" t="s">
         <v>86</v>
@@ -3833,7 +3831,7 @@
         <v>135.9</v>
       </c>
       <c r="D113" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F113" t="s">
         <v>86</v>
@@ -3859,7 +3857,7 @@
         <v>138.6</v>
       </c>
       <c r="D114" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F114" t="s">
         <v>86</v>
@@ -3885,7 +3883,7 @@
         <v>138.6</v>
       </c>
       <c r="D115" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F115" t="s">
         <v>86</v>
@@ -3911,7 +3909,7 @@
         <v>138.30000000000001</v>
       </c>
       <c r="D116" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E116" t="s">
         <v>18</v>
@@ -3940,7 +3938,7 @@
         <v>132.69999999999999</v>
       </c>
       <c r="D117" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F117" t="s">
         <v>88</v>
@@ -3966,7 +3964,7 @@
         <v>138.6</v>
       </c>
       <c r="D118" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F118" t="s">
         <v>86</v>
@@ -3992,7 +3990,7 @@
         <v>138.6</v>
       </c>
       <c r="D119" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F119" t="s">
         <v>86</v>
@@ -4018,7 +4016,7 @@
         <v>135.9</v>
       </c>
       <c r="D120" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F120" t="s">
         <v>86</v>
@@ -4044,7 +4042,7 @@
         <v>138.30000000000001</v>
       </c>
       <c r="D121" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F121" t="s">
         <v>86</v>
@@ -4070,7 +4068,7 @@
         <v>135.9</v>
       </c>
       <c r="D122" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F122" t="s">
         <v>86</v>
@@ -4096,7 +4094,7 @@
         <v>132.9</v>
       </c>
       <c r="D123" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F123" t="s">
         <v>87</v>
@@ -4122,7 +4120,7 @@
         <v>140</v>
       </c>
       <c r="D124" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F124" t="s">
         <v>90</v>
@@ -4148,7 +4146,7 @@
         <v>140</v>
       </c>
       <c r="D125" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F125" t="s">
         <v>91</v>
@@ -4174,7 +4172,7 @@
         <v>141.5</v>
       </c>
       <c r="D126" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F126" t="s">
         <v>92</v>
@@ -4200,7 +4198,7 @@
         <v>140</v>
       </c>
       <c r="D127" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F127" t="s">
         <v>92</v>
@@ -4226,7 +4224,7 @@
         <v>44.5</v>
       </c>
       <c r="D128" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F128" t="s">
         <v>95</v>
@@ -4252,7 +4250,7 @@
         <v>43.8</v>
       </c>
       <c r="D129" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F129" t="s">
         <v>96</v>
@@ -4278,7 +4276,7 @@
         <v>45</v>
       </c>
       <c r="D130" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F130" t="s">
         <v>95</v>
@@ -4304,7 +4302,7 @@
         <v>44.5</v>
       </c>
       <c r="D131" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F131" t="s">
         <v>96</v>
@@ -4330,10 +4328,10 @@
         <v>43.8</v>
       </c>
       <c r="D132" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F132" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G132" t="s">
         <v>93</v>
@@ -4356,10 +4354,10 @@
         <v>42</v>
       </c>
       <c r="D133" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F133" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G133" t="s">
         <v>93</v>
@@ -4382,10 +4380,10 @@
         <v>42</v>
       </c>
       <c r="D134" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F134" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G134" t="s">
         <v>93</v>
@@ -4408,10 +4406,10 @@
         <v>42</v>
       </c>
       <c r="D135" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F135" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G135" t="s">
         <v>93</v>
@@ -4434,7 +4432,7 @@
         <v>42</v>
       </c>
       <c r="D136" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F136" t="s">
         <v>96</v>
@@ -4460,7 +4458,7 @@
         <v>42.5</v>
       </c>
       <c r="D137" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F137" t="s">
         <v>96</v>
@@ -4486,7 +4484,7 @@
         <v>42</v>
       </c>
       <c r="D138" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F138" t="s">
         <v>96</v>
@@ -4512,7 +4510,7 @@
         <v>43</v>
       </c>
       <c r="D139" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F139" t="s">
         <v>96</v>
@@ -4538,7 +4536,7 @@
         <v>42</v>
       </c>
       <c r="D140" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F140" t="s">
         <v>96</v>
@@ -4564,16 +4562,16 @@
         <v>39.5</v>
       </c>
       <c r="D141" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F141" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G141" t="s">
         <v>93</v>
       </c>
       <c r="H141" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I141" t="s">
         <v>5</v>
@@ -4590,16 +4588,16 @@
         <v>39.5</v>
       </c>
       <c r="D142" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F142" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G142" t="s">
         <v>93</v>
       </c>
       <c r="H142" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I142" t="s">
         <v>5</v>
@@ -4616,16 +4614,16 @@
         <v>39.5</v>
       </c>
       <c r="D143" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F143" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G143" t="s">
         <v>93</v>
       </c>
       <c r="H143" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I143" t="s">
         <v>5</v>
@@ -4642,19 +4640,19 @@
         <v>38.4</v>
       </c>
       <c r="D144" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E144" t="s">
         <v>18</v>
       </c>
       <c r="F144" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G144" t="s">
         <v>93</v>
       </c>
       <c r="H144" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I144" t="s">
         <v>5</v>
@@ -4671,16 +4669,16 @@
         <v>40.5</v>
       </c>
       <c r="D145" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F145" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G145" t="s">
         <v>93</v>
       </c>
       <c r="H145" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I145" t="s">
         <v>5</v>
@@ -4697,16 +4695,16 @@
         <v>40</v>
       </c>
       <c r="D146" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F146" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G146" t="s">
         <v>93</v>
       </c>
       <c r="H146" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I146" t="s">
         <v>5</v>
@@ -4723,16 +4721,16 @@
         <v>40.200000000000003</v>
       </c>
       <c r="D147" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F147" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G147" t="s">
         <v>93</v>
       </c>
       <c r="H147" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I147" t="s">
         <v>5</v>
@@ -4749,16 +4747,16 @@
         <v>39.6</v>
       </c>
       <c r="D148" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F148" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G148" t="s">
         <v>93</v>
       </c>
       <c r="H148" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I148" t="s">
         <v>5</v>
@@ -4775,16 +4773,16 @@
         <v>39.5</v>
       </c>
       <c r="D149" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F149" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G149" t="s">
         <v>93</v>
       </c>
       <c r="H149" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I149" t="s">
         <v>5</v>
@@ -4801,16 +4799,16 @@
         <v>39.700000000000003</v>
       </c>
       <c r="D150" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F150" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G150" t="s">
         <v>93</v>
       </c>
       <c r="H150" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I150" t="s">
         <v>5</v>
@@ -4827,16 +4825,16 @@
         <v>39.799999999999997</v>
       </c>
       <c r="D151" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F151" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G151" t="s">
         <v>93</v>
       </c>
       <c r="H151" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I151" t="s">
         <v>5</v>
@@ -4853,19 +4851,19 @@
         <v>38.1</v>
       </c>
       <c r="D152" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E152" t="s">
         <v>12</v>
       </c>
       <c r="F152" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G152" t="s">
         <v>93</v>
       </c>
       <c r="H152" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I152" t="s">
         <v>5</v>
@@ -4882,19 +4880,19 @@
         <v>38.1</v>
       </c>
       <c r="D153" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E153" t="s">
         <v>12</v>
       </c>
       <c r="F153" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G153" t="s">
         <v>93</v>
       </c>
       <c r="H153" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I153" t="s">
         <v>5</v>
@@ -4911,19 +4909,19 @@
         <v>38.1</v>
       </c>
       <c r="D154" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E154" t="s">
         <v>18</v>
       </c>
       <c r="F154" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G154" t="s">
         <v>93</v>
       </c>
       <c r="H154" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I154" t="s">
         <v>5</v>
@@ -4940,19 +4938,19 @@
         <v>38.1</v>
       </c>
       <c r="D155" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E155" t="s">
         <v>19</v>
       </c>
       <c r="F155" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G155" t="s">
         <v>93</v>
       </c>
       <c r="H155" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I155" t="s">
         <v>5</v>
@@ -4969,19 +4967,19 @@
         <v>38.1</v>
       </c>
       <c r="D156" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E156" t="s">
         <v>19</v>
       </c>
       <c r="F156" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G156" t="s">
         <v>93</v>
       </c>
       <c r="H156" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I156" t="s">
         <v>5</v>
@@ -4998,19 +4996,19 @@
         <v>38.1</v>
       </c>
       <c r="D157" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E157" t="s">
         <v>19</v>
       </c>
       <c r="F157" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G157" t="s">
         <v>93</v>
       </c>
       <c r="H157" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I157" t="s">
         <v>5</v>
@@ -5027,19 +5025,19 @@
         <v>38.1</v>
       </c>
       <c r="D158" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E158" t="s">
         <v>19</v>
       </c>
       <c r="F158" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G158" t="s">
         <v>93</v>
       </c>
       <c r="H158" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I158" t="s">
         <v>5</v>
@@ -5056,19 +5054,19 @@
         <v>38.1</v>
       </c>
       <c r="D159" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E159" t="s">
         <v>19</v>
       </c>
       <c r="F159" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G159" t="s">
         <v>93</v>
       </c>
       <c r="H159" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I159" t="s">
         <v>5</v>
@@ -5085,19 +5083,19 @@
         <v>38.1</v>
       </c>
       <c r="D160" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E160" t="s">
         <v>19</v>
       </c>
       <c r="F160" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G160" t="s">
         <v>93</v>
       </c>
       <c r="H160" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I160" t="s">
         <v>5</v>
@@ -5114,19 +5112,19 @@
         <v>37.200000000000003</v>
       </c>
       <c r="D161" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E161" t="s">
         <v>18</v>
       </c>
       <c r="F161" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G161" t="s">
         <v>93</v>
       </c>
       <c r="H161" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I161" t="s">
         <v>5</v>
@@ -5143,19 +5141,19 @@
         <v>37.700000000000003</v>
       </c>
       <c r="D162" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E162" t="s">
         <v>19</v>
       </c>
       <c r="F162" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G162" t="s">
         <v>93</v>
       </c>
       <c r="H162" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I162" t="s">
         <v>5</v>
@@ -5172,19 +5170,19 @@
         <v>38.1</v>
       </c>
       <c r="D163" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E163" t="s">
         <v>19</v>
       </c>
       <c r="F163" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G163" t="s">
         <v>93</v>
       </c>
       <c r="H163" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I163" t="s">
         <v>5</v>
@@ -5201,19 +5199,19 @@
         <v>38.200000000000003</v>
       </c>
       <c r="D164" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E164" t="s">
         <v>19</v>
       </c>
       <c r="F164" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G164" t="s">
         <v>93</v>
       </c>
       <c r="H164" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I164" t="s">
         <v>5</v>
@@ -5230,19 +5228,19 @@
         <v>37.799999999999997</v>
       </c>
       <c r="D165" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E165" t="s">
         <v>18</v>
       </c>
       <c r="F165" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G165" t="s">
         <v>93</v>
       </c>
       <c r="H165" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I165" t="s">
         <v>5</v>
@@ -5259,19 +5257,19 @@
         <v>38.299999999999997</v>
       </c>
       <c r="D166" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E166" t="s">
         <v>19</v>
       </c>
       <c r="F166" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G166" t="s">
         <v>93</v>
       </c>
       <c r="H166" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I166" t="s">
         <v>5</v>
@@ -5288,16 +5286,16 @@
         <v>38.1</v>
       </c>
       <c r="D167" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F167" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G167" t="s">
         <v>93</v>
       </c>
       <c r="H167" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I167" t="s">
         <v>5</v>
@@ -5314,19 +5312,19 @@
         <v>37.700000000000003</v>
       </c>
       <c r="D168" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E168" t="s">
         <v>19</v>
       </c>
       <c r="F168" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G168" t="s">
         <v>93</v>
       </c>
       <c r="H168" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I168" t="s">
         <v>5</v>
@@ -5343,19 +5341,19 @@
         <v>37.799999999999997</v>
       </c>
       <c r="D169" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E169" t="s">
         <v>19</v>
       </c>
       <c r="F169" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G169" t="s">
         <v>93</v>
       </c>
       <c r="H169" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I169" t="s">
         <v>5</v>
@@ -5372,16 +5370,16 @@
         <v>36</v>
       </c>
       <c r="D170" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F170" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G170" t="s">
         <v>93</v>
       </c>
       <c r="H170" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I170" t="s">
         <v>5</v>
@@ -5398,16 +5396,16 @@
         <v>36.200000000000003</v>
       </c>
       <c r="D171" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F171" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G171" t="s">
         <v>93</v>
       </c>
       <c r="H171" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I171" t="s">
         <v>5</v>
@@ -5424,16 +5422,16 @@
         <v>36.5</v>
       </c>
       <c r="D172" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F172" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G172" t="s">
         <v>93</v>
       </c>
       <c r="H172" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I172" t="s">
         <v>5</v>
@@ -5450,16 +5448,16 @@
         <v>39.200000000000003</v>
       </c>
       <c r="D173" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F173" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G173" t="s">
         <v>93</v>
       </c>
       <c r="H173" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I173" t="s">
         <v>5</v>
@@ -5476,19 +5474,19 @@
         <v>38.1</v>
       </c>
       <c r="D174" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E174" t="s">
         <v>19</v>
       </c>
       <c r="F174" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G174" t="s">
         <v>93</v>
       </c>
       <c r="H174" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I174" t="s">
         <v>5</v>
@@ -5505,16 +5503,16 @@
         <v>38.299999999999997</v>
       </c>
       <c r="D175" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F175" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G175" t="s">
         <v>93</v>
       </c>
       <c r="H175" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I175" t="s">
         <v>5</v>
@@ -5531,19 +5529,19 @@
         <v>38</v>
       </c>
       <c r="D176" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E176" t="s">
         <v>19</v>
       </c>
       <c r="F176" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G176" t="s">
         <v>93</v>
       </c>
       <c r="H176" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I176" t="s">
         <v>5</v>
@@ -5560,16 +5558,16 @@
         <v>38.200000000000003</v>
       </c>
       <c r="D177" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F177" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G177" t="s">
         <v>93</v>
       </c>
       <c r="H177" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I177" t="s">
         <v>5</v>
@@ -5586,7 +5584,7 @@
         <v>38</v>
       </c>
       <c r="D178" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E178" t="s">
         <v>12</v>
@@ -5598,7 +5596,7 @@
         <v>93</v>
       </c>
       <c r="H178" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I178" t="s">
         <v>5</v>
@@ -5615,16 +5613,16 @@
         <v>36</v>
       </c>
       <c r="D179" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F179" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G179" t="s">
         <v>93</v>
       </c>
       <c r="H179" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I179" t="s">
         <v>47</v>
@@ -5641,16 +5639,16 @@
         <v>36</v>
       </c>
       <c r="D180" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F180" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G180" t="s">
         <v>93</v>
       </c>
       <c r="H180" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I180" t="s">
         <v>48</v>
@@ -5667,16 +5665,16 @@
         <v>36</v>
       </c>
       <c r="D181" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F181" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G181" t="s">
         <v>93</v>
       </c>
       <c r="H181" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I181" t="s">
         <v>49</v>
@@ -5693,16 +5691,16 @@
         <v>36</v>
       </c>
       <c r="D182" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F182" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G182" t="s">
         <v>93</v>
       </c>
       <c r="H182" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I182" t="s">
         <v>50</v>
@@ -5719,16 +5717,16 @@
         <v>36</v>
       </c>
       <c r="D183" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F183" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G183" t="s">
         <v>93</v>
       </c>
       <c r="H183" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I183" t="s">
         <v>51</v>
@@ -5745,16 +5743,16 @@
         <v>36</v>
       </c>
       <c r="D184" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F184" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G184" t="s">
         <v>93</v>
       </c>
       <c r="H184" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I184" t="s">
         <v>53</v>
@@ -5771,19 +5769,19 @@
         <v>33</v>
       </c>
       <c r="D185" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E185" t="s">
         <v>18</v>
       </c>
       <c r="F185" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G185" t="s">
         <v>93</v>
       </c>
       <c r="H185" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I185" t="s">
         <v>54</v>
@@ -5800,16 +5798,16 @@
         <v>35</v>
       </c>
       <c r="D186" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F186" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G186" t="s">
         <v>93</v>
       </c>
       <c r="H186" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I186" t="s">
         <v>55</v>
@@ -5826,19 +5824,19 @@
         <v>33.6</v>
       </c>
       <c r="D187" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E187" t="s">
         <v>18</v>
       </c>
       <c r="F187" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G187" t="s">
         <v>93</v>
       </c>
       <c r="H187" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I187" t="s">
         <v>56</v>
@@ -5855,16 +5853,16 @@
         <v>33.1</v>
       </c>
       <c r="D188" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F188" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G188" t="s">
         <v>93</v>
       </c>
       <c r="H188" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I188" t="s">
         <v>57</v>
@@ -5881,16 +5879,16 @@
         <v>35.6</v>
       </c>
       <c r="D189" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F189" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G189" t="s">
         <v>93</v>
       </c>
       <c r="H189" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I189" t="s">
         <v>66</v>
@@ -5907,19 +5905,19 @@
         <v>83.5</v>
       </c>
       <c r="D190" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F190" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="G190" t="s">
+        <v>123</v>
+      </c>
+      <c r="H190" t="s">
+        <v>133</v>
+      </c>
+      <c r="I190" t="s">
         <v>122</v>
-      </c>
-      <c r="G190" t="s">
-        <v>124</v>
-      </c>
-      <c r="H190" t="s">
-        <v>134</v>
-      </c>
-      <c r="I190" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="191" spans="1:9">
@@ -5933,19 +5931,19 @@
         <v>76</v>
       </c>
       <c r="D191" t="s">
+        <v>125</v>
+      </c>
+      <c r="F191" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="F191" s="2" t="s">
-        <v>127</v>
-      </c>
       <c r="G191" t="s">
+        <v>123</v>
+      </c>
+      <c r="H191" t="s">
         <v>124</v>
       </c>
-      <c r="H191" t="s">
-        <v>125</v>
-      </c>
       <c r="I191" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="192" spans="1:9">
@@ -5959,19 +5957,19 @@
         <v>91.1</v>
       </c>
       <c r="D192" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F192" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G192" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H192" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I192" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="193" spans="1:9">
@@ -5985,19 +5983,19 @@
         <v>79.7</v>
       </c>
       <c r="D193" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F193" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G193" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H193" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I193" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="194" spans="1:9">
@@ -6011,19 +6009,19 @@
         <v>77.3</v>
       </c>
       <c r="D194" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F194" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G194" t="s">
+        <v>123</v>
+      </c>
+      <c r="H194" t="s">
         <v>124</v>
       </c>
-      <c r="H194" t="s">
-        <v>125</v>
-      </c>
       <c r="I194" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="195" spans="1:9">
@@ -6037,19 +6035,19 @@
         <v>87.5</v>
       </c>
       <c r="D195" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F195" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G195" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H195" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I195" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="196" spans="1:9">
@@ -6063,19 +6061,19 @@
         <v>95.5</v>
       </c>
       <c r="D196" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F196" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G196" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H196" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I196" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="197" spans="1:9">
@@ -6089,19 +6087,19 @@
         <v>85.9</v>
       </c>
       <c r="D197" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F197" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G197" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H197" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I197" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="198" spans="1:9">
@@ -6115,17 +6113,17 @@
         <v>86.1</v>
       </c>
       <c r="D198" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F198" s="2"/>
       <c r="G198" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H198" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I198" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="199" spans="1:9">
@@ -6139,16 +6137,16 @@
         <v>87.5</v>
       </c>
       <c r="D199" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G199" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H199" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I199" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="200" spans="1:9">
@@ -6164,19 +6162,19 @@
         <v>-39.104548110000003</v>
       </c>
       <c r="D200" t="s">
+        <v>138</v>
+      </c>
+      <c r="F200" t="s">
         <v>139</v>
       </c>
-      <c r="F200" t="s">
+      <c r="G200" t="s">
         <v>140</v>
       </c>
-      <c r="G200" t="s">
+      <c r="H200" t="s">
         <v>141</v>
       </c>
-      <c r="H200" t="s">
-        <v>142</v>
-      </c>
       <c r="I200" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="201" spans="1:9">
@@ -6192,19 +6190,19 @@
         <v>-38.531135749999997</v>
       </c>
       <c r="D201" t="s">
+        <v>138</v>
+      </c>
+      <c r="F201" t="s">
         <v>139</v>
       </c>
-      <c r="F201" t="s">
+      <c r="G201" t="s">
         <v>140</v>
       </c>
-      <c r="G201" t="s">
-        <v>141</v>
-      </c>
       <c r="H201" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I201" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="202" spans="1:9">
@@ -6220,19 +6218,19 @@
         <v>-38.6166883</v>
       </c>
       <c r="D202" t="s">
+        <v>138</v>
+      </c>
+      <c r="F202" t="s">
         <v>139</v>
       </c>
-      <c r="F202" t="s">
+      <c r="G202" t="s">
         <v>140</v>
       </c>
-      <c r="G202" t="s">
-        <v>141</v>
-      </c>
       <c r="H202" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I202" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="203" spans="1:9">
@@ -6248,19 +6246,19 @@
         <v>-38.369071699999999</v>
       </c>
       <c r="D203" t="s">
+        <v>138</v>
+      </c>
+      <c r="F203" t="s">
         <v>139</v>
       </c>
-      <c r="F203" t="s">
+      <c r="G203" t="s">
         <v>140</v>
       </c>
-      <c r="G203" t="s">
-        <v>141</v>
-      </c>
       <c r="H203" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I203" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="204" spans="1:9">
@@ -6275,19 +6273,19 @@
         <v>-39.104548110000003</v>
       </c>
       <c r="D204" t="s">
+        <v>138</v>
+      </c>
+      <c r="F204" t="s">
         <v>139</v>
       </c>
-      <c r="F204" t="s">
+      <c r="G204" t="s">
         <v>140</v>
       </c>
-      <c r="G204" t="s">
+      <c r="H204" t="s">
         <v>141</v>
       </c>
-      <c r="H204" t="s">
-        <v>142</v>
-      </c>
       <c r="I204" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="205" spans="1:9">
@@ -6302,19 +6300,19 @@
         <v>-39.48480979</v>
       </c>
       <c r="D205" t="s">
+        <v>138</v>
+      </c>
+      <c r="F205" t="s">
         <v>139</v>
       </c>
-      <c r="F205" t="s">
+      <c r="G205" t="s">
         <v>140</v>
       </c>
-      <c r="G205" t="s">
-        <v>141</v>
-      </c>
       <c r="H205" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I205" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="206" spans="1:9">
@@ -6329,19 +6327,19 @@
         <v>-38.369071699999999</v>
       </c>
       <c r="D206" t="s">
+        <v>138</v>
+      </c>
+      <c r="F206" t="s">
         <v>139</v>
       </c>
-      <c r="F206" t="s">
+      <c r="G206" t="s">
         <v>140</v>
       </c>
-      <c r="G206" t="s">
-        <v>141</v>
-      </c>
       <c r="H206" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I206" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="207" spans="1:9">
@@ -6356,19 +6354,19 @@
         <v>-39.104548110000003</v>
       </c>
       <c r="D207" t="s">
+        <v>138</v>
+      </c>
+      <c r="F207" t="s">
         <v>139</v>
       </c>
-      <c r="F207" t="s">
+      <c r="G207" t="s">
         <v>140</v>
       </c>
-      <c r="G207" t="s">
-        <v>141</v>
-      </c>
       <c r="H207" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I207" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="208" spans="1:9">
@@ -6383,19 +6381,19 @@
         <v>-38.369071699999999</v>
       </c>
       <c r="D208" t="s">
+        <v>138</v>
+      </c>
+      <c r="F208" t="s">
         <v>139</v>
       </c>
-      <c r="F208" t="s">
+      <c r="G208" t="s">
         <v>140</v>
       </c>
-      <c r="G208" t="s">
-        <v>141</v>
-      </c>
       <c r="H208" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I208" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="209" spans="1:9">
@@ -6410,19 +6408,19 @@
         <v>-41.243539550000001</v>
       </c>
       <c r="D209" t="s">
+        <v>138</v>
+      </c>
+      <c r="F209" t="s">
         <v>139</v>
       </c>
-      <c r="F209" t="s">
+      <c r="G209" t="s">
         <v>140</v>
       </c>
-      <c r="G209" t="s">
-        <v>141</v>
-      </c>
       <c r="H209" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I209" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed Tohoku and 1938 event extent error
</commit_message>
<xml_diff>
--- a/data_compilation.xlsx
+++ b/data_compilation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/albamarrodriguezpadilla/Downloads/paleoseismology_subduction-main/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B5BA4C4-20FF-B448-AEFB-446668F63447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E12520DD-28B7-A04C-B4FB-5FD6B557B05C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{0C72CEA8-103F-664E-BFC3-8082C479B46F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="137">
   <si>
     <t>Year</t>
   </si>
@@ -179,39 +179,9 @@
     <t>Noquet et al., 2016</t>
   </si>
   <si>
-    <t>Philibosian and Metlzner, 2021</t>
-  </si>
-  <si>
-    <t>Philibosian and Metlzner, 2022</t>
-  </si>
-  <si>
-    <t>Philibosian and Metlzner, 2023</t>
-  </si>
-  <si>
-    <t>Philibosian and Metlzner, 2024</t>
-  </si>
-  <si>
-    <t>Philibosian and Metlzner, 2025</t>
-  </si>
-  <si>
     <t>Chiclayo Segment</t>
   </si>
   <si>
-    <t>Philibosian and Metlzner, 2026</t>
-  </si>
-  <si>
-    <t>Philibosian and Metlzner, 2027</t>
-  </si>
-  <si>
-    <t>Philibosian and Metlzner, 2028</t>
-  </si>
-  <si>
-    <t>Philibosian and Metlzner, 2029</t>
-  </si>
-  <si>
-    <t>Philibosian and Metlzner, 2030</t>
-  </si>
-  <si>
     <t>Dorbath et al., 1990</t>
   </si>
   <si>
@@ -234,9 +204,6 @@
   </si>
   <si>
     <t>Iquique Segment</t>
-  </si>
-  <si>
-    <t>Philibosian and Metlzner, 2031</t>
   </si>
   <si>
     <t>Comte and Pardo, 1991</t>
@@ -865,19 +832,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="C1" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="D1" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="E1" t="s">
         <v>1</v>
       </c>
       <c r="F1" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="G1" t="s">
         <v>2</v>
@@ -923,7 +890,7 @@
         <v>2.5</v>
       </c>
       <c r="D3" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F3" t="s">
         <v>6</v>
@@ -949,7 +916,7 @@
         <v>3.5</v>
       </c>
       <c r="D4" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F4" t="s">
         <v>7</v>
@@ -975,7 +942,7 @@
         <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F5" t="s">
         <v>8</v>
@@ -1001,7 +968,7 @@
         <v>6.6</v>
       </c>
       <c r="D6" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F6" t="s">
         <v>9</v>
@@ -1027,7 +994,7 @@
         <v>8.6999999999999993</v>
       </c>
       <c r="D7" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F7" t="s">
         <v>10</v>
@@ -1053,7 +1020,7 @@
         <v>11.4</v>
       </c>
       <c r="D8" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F8" t="s">
         <v>11</v>
@@ -1079,7 +1046,7 @@
         <v>2.5</v>
       </c>
       <c r="D9" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E9" t="s">
         <v>12</v>
@@ -1108,7 +1075,7 @@
         <v>2.4</v>
       </c>
       <c r="D10" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F10" t="s">
         <v>15</v>
@@ -1134,7 +1101,7 @@
         <v>2.5</v>
       </c>
       <c r="D11" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F11" t="s">
         <v>15</v>
@@ -1160,7 +1127,7 @@
         <v>0</v>
       </c>
       <c r="D12" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F12" t="s">
         <v>20</v>
@@ -1186,7 +1153,7 @@
         <v>17</v>
       </c>
       <c r="D13" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F13" t="s">
         <v>20</v>
@@ -1212,7 +1179,7 @@
         <v>0.8</v>
       </c>
       <c r="D14" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F14" t="s">
         <v>21</v>
@@ -1238,7 +1205,7 @@
         <v>0</v>
       </c>
       <c r="D15" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F15" t="s">
         <v>21</v>
@@ -1264,7 +1231,7 @@
         <v>0.5</v>
       </c>
       <c r="D16" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E16" t="s">
         <v>18</v>
@@ -1293,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="D17" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F17" t="s">
         <v>23</v>
@@ -1319,7 +1286,7 @@
         <v>1.7</v>
       </c>
       <c r="D18" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E18" t="s">
         <v>19</v>
@@ -1348,7 +1315,7 @@
         <v>-0.5</v>
       </c>
       <c r="D19" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F19" t="s">
         <v>26</v>
@@ -1374,7 +1341,7 @@
         <v>5</v>
       </c>
       <c r="D20" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F20" t="s">
         <v>27</v>
@@ -1400,7 +1367,7 @@
         <v>-3.6</v>
       </c>
       <c r="D21" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E21" t="s">
         <v>18</v>
@@ -1429,7 +1396,7 @@
         <v>-4.5</v>
       </c>
       <c r="D22" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F22" t="s">
         <v>30</v>
@@ -1455,7 +1422,7 @@
         <v>-3.5</v>
       </c>
       <c r="D23" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F23" t="s">
         <v>30</v>
@@ -1481,7 +1448,7 @@
         <v>-3.5</v>
       </c>
       <c r="D24" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F24" t="s">
         <v>31</v>
@@ -1507,7 +1474,7 @@
         <v>-3.7</v>
       </c>
       <c r="D25" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F25" t="s">
         <v>31</v>
@@ -1533,7 +1500,7 @@
         <v>-4</v>
       </c>
       <c r="D26" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E26" t="s">
         <v>19</v>
@@ -1562,7 +1529,7 @@
         <v>-2.5</v>
       </c>
       <c r="D27" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F27" t="s">
         <v>31</v>
@@ -1588,7 +1555,7 @@
         <v>-4.5</v>
       </c>
       <c r="D28" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F28" t="s">
         <v>31</v>
@@ -1614,7 +1581,7 @@
         <v>-3.4</v>
       </c>
       <c r="D29" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F29" t="s">
         <v>32</v>
@@ -1640,7 +1607,7 @@
         <v>-4.5</v>
       </c>
       <c r="D30" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F30" t="s">
         <v>32</v>
@@ -1666,7 +1633,7 @@
         <v>-4.5</v>
       </c>
       <c r="D31" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F31" t="s">
         <v>33</v>
@@ -1692,7 +1659,7 @@
         <v>-2.8</v>
       </c>
       <c r="D32" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E32" t="s">
         <v>19</v>
@@ -1721,7 +1688,7 @@
         <v>-2</v>
       </c>
       <c r="D33" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E33" t="s">
         <v>19</v>
@@ -1750,7 +1717,7 @@
         <v>-2.7</v>
       </c>
       <c r="D34" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F34" t="s">
         <v>36</v>
@@ -1776,7 +1743,7 @@
         <v>-4</v>
       </c>
       <c r="D35" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E35" t="s">
         <v>18</v>
@@ -1805,7 +1772,7 @@
         <v>-5.7</v>
       </c>
       <c r="D36" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F36" t="s">
         <v>39</v>
@@ -1831,7 +1798,7 @@
         <v>-0.5</v>
       </c>
       <c r="D37" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F37" t="s">
         <v>42</v>
@@ -1857,7 +1824,7 @@
         <v>0</v>
       </c>
       <c r="D38" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F38" t="s">
         <v>44</v>
@@ -1883,7 +1850,7 @@
         <v>0</v>
       </c>
       <c r="D39" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F39" t="s">
         <v>42</v>
@@ -1909,7 +1876,7 @@
         <v>-0.5</v>
       </c>
       <c r="D40" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F40" t="s">
         <v>42</v>
@@ -1935,7 +1902,7 @@
         <v>1.2</v>
       </c>
       <c r="D41" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F41" t="s">
         <v>42</v>
@@ -1961,7 +1928,7 @@
         <v>1.7</v>
       </c>
       <c r="D42" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F42" t="s">
         <v>42</v>
@@ -1987,7 +1954,7 @@
         <v>-0.6</v>
       </c>
       <c r="D43" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F43" t="s">
         <v>42</v>
@@ -2013,7 +1980,7 @@
         <v>-0.5</v>
       </c>
       <c r="D44" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F44" t="s">
         <v>46</v>
@@ -2039,16 +2006,16 @@
         <v>-8.5</v>
       </c>
       <c r="D45" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F45" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="G45" t="s">
         <v>45</v>
       </c>
       <c r="H45" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="I45" t="s">
         <v>5</v>
@@ -2065,16 +2032,16 @@
         <v>-4.5</v>
       </c>
       <c r="D46" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F46" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="G46" t="s">
         <v>45</v>
       </c>
       <c r="H46" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="I46" t="s">
         <v>5</v>
@@ -2091,16 +2058,16 @@
         <v>-5</v>
       </c>
       <c r="D47" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F47" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="G47" t="s">
         <v>45</v>
       </c>
       <c r="H47" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="I47" t="s">
         <v>5</v>
@@ -2117,19 +2084,19 @@
         <v>-7.5</v>
       </c>
       <c r="D48" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E48" t="s">
         <v>18</v>
       </c>
       <c r="F48" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G48" t="s">
         <v>45</v>
       </c>
       <c r="H48" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="I48" t="s">
         <v>5</v>
@@ -2146,19 +2113,19 @@
         <v>-10.199999999999999</v>
       </c>
       <c r="D49" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E49" t="s">
         <v>18</v>
       </c>
       <c r="F49" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G49" t="s">
         <v>45</v>
       </c>
       <c r="H49" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="I49" t="s">
         <v>5</v>
@@ -2175,16 +2142,16 @@
         <v>-13.7</v>
       </c>
       <c r="D50" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F50" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="G50" t="s">
         <v>45</v>
       </c>
       <c r="H50" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="I50" t="s">
         <v>5</v>
@@ -2201,16 +2168,16 @@
         <v>-14.8</v>
       </c>
       <c r="D51" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F51" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="G51" t="s">
         <v>45</v>
       </c>
       <c r="H51" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="I51" t="s">
         <v>5</v>
@@ -2227,16 +2194,16 @@
         <v>-11.5</v>
       </c>
       <c r="D52" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F52" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="G52" t="s">
         <v>45</v>
       </c>
       <c r="H52" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="I52" t="s">
         <v>5</v>
@@ -2253,16 +2220,16 @@
         <v>-15.2</v>
       </c>
       <c r="D53" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F53" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="G53" t="s">
         <v>45</v>
       </c>
       <c r="H53" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="I53" t="s">
         <v>5</v>
@@ -2279,16 +2246,16 @@
         <v>-13.5</v>
       </c>
       <c r="D54" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F54" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="G54" t="s">
         <v>45</v>
       </c>
       <c r="H54" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="I54" t="s">
         <v>5</v>
@@ -2305,16 +2272,16 @@
         <v>-11.5</v>
       </c>
       <c r="D55" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F55" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G55" t="s">
         <v>45</v>
       </c>
       <c r="H55" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="I55" t="s">
         <v>5</v>
@@ -2331,16 +2298,16 @@
         <v>-11.2</v>
       </c>
       <c r="D56" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F56" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G56" t="s">
         <v>45</v>
       </c>
       <c r="H56" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="I56" t="s">
         <v>5</v>
@@ -2357,16 +2324,16 @@
         <v>-13.5</v>
       </c>
       <c r="D57" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F57" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G57" t="s">
         <v>45</v>
       </c>
       <c r="H57" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="I57" t="s">
         <v>5</v>
@@ -2383,16 +2350,16 @@
         <v>-14</v>
       </c>
       <c r="D58" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F58" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G58" t="s">
         <v>45</v>
       </c>
       <c r="H58" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="I58" t="s">
         <v>5</v>
@@ -2409,16 +2376,16 @@
         <v>-17</v>
       </c>
       <c r="D59" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F59" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="G59" t="s">
         <v>45</v>
       </c>
       <c r="H59" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="I59" t="s">
         <v>5</v>
@@ -2435,16 +2402,16 @@
         <v>-18.2</v>
       </c>
       <c r="D60" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F60" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="G60" t="s">
         <v>45</v>
       </c>
       <c r="H60" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="I60" t="s">
         <v>5</v>
@@ -2461,16 +2428,16 @@
         <v>-17.5</v>
       </c>
       <c r="D61" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F61" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="G61" t="s">
         <v>45</v>
       </c>
       <c r="H61" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="I61" t="s">
         <v>5</v>
@@ -2487,16 +2454,16 @@
         <v>-18</v>
       </c>
       <c r="D62" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F62" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="G62" t="s">
         <v>45</v>
       </c>
       <c r="H62" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="I62" t="s">
         <v>5</v>
@@ -2513,16 +2480,16 @@
         <v>-18</v>
       </c>
       <c r="D63" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F63" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="G63" t="s">
         <v>45</v>
       </c>
       <c r="H63" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="I63" t="s">
         <v>5</v>
@@ -2539,16 +2506,16 @@
         <v>-18.5</v>
       </c>
       <c r="D64" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F64" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="G64" t="s">
         <v>45</v>
       </c>
       <c r="H64" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="I64" t="s">
         <v>5</v>
@@ -2565,16 +2532,16 @@
         <v>-15.8</v>
       </c>
       <c r="D65" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F65" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G65" t="s">
         <v>45</v>
       </c>
       <c r="H65" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="I65" t="s">
         <v>5</v>
@@ -2591,16 +2558,16 @@
         <v>-15.5</v>
       </c>
       <c r="D66" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F66" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G66" t="s">
         <v>45</v>
       </c>
       <c r="H66" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="I66" t="s">
         <v>5</v>
@@ -2617,16 +2584,16 @@
         <v>-17.2</v>
       </c>
       <c r="D67" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F67" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G67" t="s">
         <v>45</v>
       </c>
       <c r="H67" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="I67" t="s">
         <v>5</v>
@@ -2643,16 +2610,16 @@
         <v>-18</v>
       </c>
       <c r="D68" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F68" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G68" t="s">
         <v>45</v>
       </c>
       <c r="H68" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="I68" t="s">
         <v>5</v>
@@ -2669,16 +2636,16 @@
         <v>-20</v>
       </c>
       <c r="D69" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F69" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="G69" t="s">
         <v>45</v>
       </c>
       <c r="H69" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="I69" t="s">
         <v>5</v>
@@ -2695,16 +2662,16 @@
         <v>-19</v>
       </c>
       <c r="D70" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F70" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="G70" t="s">
         <v>45</v>
       </c>
       <c r="H70" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="I70" t="s">
         <v>5</v>
@@ -2721,16 +2688,16 @@
         <v>-21.5</v>
       </c>
       <c r="D71" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F71" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="G71" t="s">
         <v>45</v>
       </c>
       <c r="H71" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="I71" t="s">
         <v>5</v>
@@ -2747,16 +2714,16 @@
         <v>-19.399999999999999</v>
       </c>
       <c r="D72" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F72" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="G72" t="s">
         <v>45</v>
       </c>
       <c r="H72" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="I72" t="s">
         <v>5</v>
@@ -2773,16 +2740,16 @@
         <v>-22.5</v>
       </c>
       <c r="D73" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F73" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="G73" t="s">
         <v>45</v>
       </c>
       <c r="H73" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="I73" t="s">
         <v>5</v>
@@ -2799,16 +2766,16 @@
         <v>-20</v>
       </c>
       <c r="D74" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F74" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="G74" t="s">
         <v>45</v>
       </c>
       <c r="H74" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="I74" t="s">
         <v>5</v>
@@ -2825,16 +2792,16 @@
         <v>-20.7</v>
       </c>
       <c r="D75" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F75" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="G75" t="s">
         <v>45</v>
       </c>
       <c r="H75" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="I75" t="s">
         <v>5</v>
@@ -2851,16 +2818,16 @@
         <v>-23</v>
       </c>
       <c r="D76" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F76" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="G76" t="s">
         <v>45</v>
       </c>
       <c r="H76" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="I76" t="s">
         <v>5</v>
@@ -2877,16 +2844,16 @@
         <v>-20.5</v>
       </c>
       <c r="D77" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F77" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="G77" t="s">
         <v>45</v>
       </c>
       <c r="H77" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="I77" t="s">
         <v>5</v>
@@ -2903,16 +2870,16 @@
         <v>-23.2</v>
       </c>
       <c r="D78" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F78" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G78" t="s">
         <v>45</v>
       </c>
       <c r="H78" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="I78" t="s">
         <v>5</v>
@@ -2929,16 +2896,16 @@
         <v>-20.3</v>
       </c>
       <c r="D79" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F79" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="G79" t="s">
         <v>45</v>
       </c>
       <c r="H79" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="I79" t="s">
         <v>5</v>
@@ -2955,16 +2922,16 @@
         <v>-20.7</v>
       </c>
       <c r="D80" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F80" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="G80" t="s">
         <v>45</v>
       </c>
       <c r="H80" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="I80" t="s">
         <v>5</v>
@@ -2981,16 +2948,16 @@
         <v>-25</v>
       </c>
       <c r="D81" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F81" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G81" t="s">
         <v>45</v>
       </c>
       <c r="H81" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="I81" t="s">
         <v>5</v>
@@ -3007,19 +2974,19 @@
         <v>-28.5</v>
       </c>
       <c r="D82" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E82" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="F82" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="G82" t="s">
         <v>45</v>
       </c>
       <c r="H82" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="I82" t="s">
         <v>5</v>
@@ -3036,19 +3003,19 @@
         <v>-30</v>
       </c>
       <c r="D83" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E83" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="F83" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="G83" t="s">
         <v>45</v>
       </c>
       <c r="H83" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="I83" t="s">
         <v>5</v>
@@ -3065,16 +3032,16 @@
         <v>-26.5</v>
       </c>
       <c r="D84" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F84" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="G84" t="s">
         <v>45</v>
       </c>
       <c r="H84" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="I84" t="s">
         <v>5</v>
@@ -3091,16 +3058,16 @@
         <v>-30.2</v>
       </c>
       <c r="D85" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F85" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="G85" t="s">
         <v>45</v>
       </c>
       <c r="H85" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="I85" t="s">
         <v>5</v>
@@ -3117,16 +3084,16 @@
         <v>-34</v>
       </c>
       <c r="D86" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F86" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="G86" t="s">
         <v>45</v>
       </c>
       <c r="H86" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="I86" t="s">
         <v>5</v>
@@ -3143,16 +3110,16 @@
         <v>-35</v>
       </c>
       <c r="D87" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F87" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="G87" t="s">
         <v>45</v>
       </c>
       <c r="H87" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="I87" t="s">
         <v>5</v>
@@ -3169,16 +3136,16 @@
         <v>-36</v>
       </c>
       <c r="D88" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F88" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="G88" t="s">
         <v>45</v>
       </c>
       <c r="H88" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="I88" t="s">
         <v>5</v>
@@ -3195,16 +3162,16 @@
         <v>-33.700000000000003</v>
       </c>
       <c r="D89" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F89" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="G89" t="s">
         <v>45</v>
       </c>
       <c r="H89" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="I89" t="s">
         <v>5</v>
@@ -3221,16 +3188,16 @@
         <v>-33.700000000000003</v>
       </c>
       <c r="D90" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F90" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="G90" t="s">
         <v>45</v>
       </c>
       <c r="H90" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="I90" t="s">
         <v>5</v>
@@ -3247,16 +3214,16 @@
         <v>-33</v>
       </c>
       <c r="D91" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F91" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="G91" t="s">
         <v>45</v>
       </c>
       <c r="H91" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="I91" t="s">
         <v>5</v>
@@ -3273,16 +3240,16 @@
         <v>-32</v>
       </c>
       <c r="D92" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F92" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="G92" t="s">
         <v>45</v>
       </c>
       <c r="H92" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="I92" t="s">
         <v>5</v>
@@ -3299,16 +3266,16 @@
         <v>-35</v>
       </c>
       <c r="D93" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F93" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="G93" t="s">
         <v>45</v>
       </c>
       <c r="H93" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="I93" t="s">
         <v>5</v>
@@ -3325,16 +3292,16 @@
         <v>-32</v>
       </c>
       <c r="D94" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F94" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="G94" t="s">
         <v>45</v>
       </c>
       <c r="H94" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="I94" t="s">
         <v>5</v>
@@ -3351,16 +3318,16 @@
         <v>-33</v>
       </c>
       <c r="D95" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F95" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="G95" t="s">
         <v>45</v>
       </c>
       <c r="H95" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="I95" t="s">
         <v>5</v>
@@ -3377,16 +3344,16 @@
         <v>-34.5</v>
       </c>
       <c r="D96" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F96" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="G96" t="s">
         <v>45</v>
       </c>
       <c r="H96" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="I96" t="s">
         <v>5</v>
@@ -3403,16 +3370,16 @@
         <v>-32</v>
       </c>
       <c r="D97" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F97" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="G97" t="s">
         <v>45</v>
       </c>
       <c r="H97" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="I97" t="s">
         <v>5</v>
@@ -3429,16 +3396,16 @@
         <v>-38</v>
       </c>
       <c r="D98" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F98" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="G98" t="s">
         <v>45</v>
       </c>
       <c r="H98" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="I98" t="s">
         <v>5</v>
@@ -3455,16 +3422,16 @@
         <v>-38.5</v>
       </c>
       <c r="D99" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F99" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="G99" t="s">
         <v>45</v>
       </c>
       <c r="H99" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="I99" t="s">
         <v>5</v>
@@ -3481,16 +3448,16 @@
         <v>-39</v>
       </c>
       <c r="D100" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F100" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="G100" t="s">
         <v>45</v>
       </c>
       <c r="H100" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="I100" t="s">
         <v>5</v>
@@ -3507,16 +3474,16 @@
         <v>-38.5</v>
       </c>
       <c r="D101" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F101" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="G101" t="s">
         <v>45</v>
       </c>
       <c r="H101" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="I101" t="s">
         <v>5</v>
@@ -3533,16 +3500,16 @@
         <v>-36</v>
       </c>
       <c r="D102" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F102" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="G102" t="s">
         <v>45</v>
       </c>
       <c r="H102" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="I102" t="s">
         <v>5</v>
@@ -3559,16 +3526,16 @@
         <v>-38</v>
       </c>
       <c r="D103" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F103" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="G103" t="s">
         <v>45</v>
       </c>
       <c r="H103" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="I103" t="s">
         <v>5</v>
@@ -3585,16 +3552,16 @@
         <v>-38.5</v>
       </c>
       <c r="D104" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F104" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="G104" t="s">
         <v>45</v>
       </c>
       <c r="H104" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="I104" t="s">
         <v>5</v>
@@ -3611,19 +3578,19 @@
         <v>-46</v>
       </c>
       <c r="D105" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E105" t="s">
         <v>12</v>
       </c>
       <c r="F105" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="G105" t="s">
         <v>45</v>
       </c>
       <c r="H105" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="I105" t="s">
         <v>5</v>
@@ -3640,19 +3607,19 @@
         <v>-46</v>
       </c>
       <c r="D106" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E106" t="s">
         <v>19</v>
       </c>
       <c r="F106" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="G106" t="s">
         <v>45</v>
       </c>
       <c r="H106" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="I106" t="s">
         <v>5</v>
@@ -3669,19 +3636,19 @@
         <v>-46</v>
       </c>
       <c r="D107" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E107" t="s">
         <v>12</v>
       </c>
       <c r="F107" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="G107" t="s">
         <v>45</v>
       </c>
       <c r="H107" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="I107" t="s">
         <v>5</v>
@@ -3698,19 +3665,19 @@
         <v>-46</v>
       </c>
       <c r="D108" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E108" t="s">
         <v>12</v>
       </c>
       <c r="F108" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="G108" t="s">
         <v>45</v>
       </c>
       <c r="H108" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="I108" t="s">
         <v>5</v>
@@ -3727,16 +3694,16 @@
         <v>-43.8</v>
       </c>
       <c r="D109" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F109" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="G109" t="s">
         <v>45</v>
       </c>
       <c r="H109" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="I109" t="s">
         <v>5</v>
@@ -3753,16 +3720,16 @@
         <v>138.6</v>
       </c>
       <c r="D110" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F110" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="G110" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H110" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="I110" t="s">
         <v>5</v>
@@ -3779,16 +3746,16 @@
         <v>138.6</v>
       </c>
       <c r="D111" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F111" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="G111" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H111" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="I111" t="s">
         <v>5</v>
@@ -3805,16 +3772,16 @@
         <v>138.30000000000001</v>
       </c>
       <c r="D112" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F112" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="G112" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H112" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="I112" t="s">
         <v>5</v>
@@ -3831,16 +3798,16 @@
         <v>135.9</v>
       </c>
       <c r="D113" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F113" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="G113" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H113" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="I113" t="s">
         <v>5</v>
@@ -3857,16 +3824,16 @@
         <v>138.6</v>
       </c>
       <c r="D114" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F114" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="G114" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H114" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="I114" t="s">
         <v>5</v>
@@ -3883,16 +3850,16 @@
         <v>138.6</v>
       </c>
       <c r="D115" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F115" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="G115" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H115" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="I115" t="s">
         <v>5</v>
@@ -3909,19 +3876,19 @@
         <v>138.30000000000001</v>
       </c>
       <c r="D116" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E116" t="s">
         <v>18</v>
       </c>
       <c r="F116" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="G116" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H116" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="I116" t="s">
         <v>5</v>
@@ -3938,16 +3905,16 @@
         <v>132.69999999999999</v>
       </c>
       <c r="D117" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F117" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="G117" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H117" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="I117" t="s">
         <v>5</v>
@@ -3964,16 +3931,16 @@
         <v>138.6</v>
       </c>
       <c r="D118" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F118" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="G118" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H118" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="I118" t="s">
         <v>5</v>
@@ -3990,16 +3957,16 @@
         <v>138.6</v>
       </c>
       <c r="D119" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F119" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="G119" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H119" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="I119" t="s">
         <v>5</v>
@@ -4016,16 +3983,16 @@
         <v>135.9</v>
       </c>
       <c r="D120" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F120" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="G120" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H120" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="I120" t="s">
         <v>5</v>
@@ -4042,16 +4009,16 @@
         <v>138.30000000000001</v>
       </c>
       <c r="D121" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F121" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="G121" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H121" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="I121" t="s">
         <v>5</v>
@@ -4068,16 +4035,16 @@
         <v>135.9</v>
       </c>
       <c r="D122" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F122" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="G122" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H122" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="I122" t="s">
         <v>5</v>
@@ -4094,16 +4061,16 @@
         <v>132.9</v>
       </c>
       <c r="D123" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F123" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="G123" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H123" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="I123" t="s">
         <v>5</v>
@@ -4120,16 +4087,16 @@
         <v>140</v>
       </c>
       <c r="D124" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F124" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="G124" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H124" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="I124" t="s">
         <v>5</v>
@@ -4146,16 +4113,16 @@
         <v>140</v>
       </c>
       <c r="D125" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F125" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="G125" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H125" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="I125" t="s">
         <v>5</v>
@@ -4172,16 +4139,16 @@
         <v>141.5</v>
       </c>
       <c r="D126" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F126" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G126" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H126" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="I126" t="s">
         <v>5</v>
@@ -4198,16 +4165,16 @@
         <v>140</v>
       </c>
       <c r="D127" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F127" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G127" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="H127" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="I127" t="s">
         <v>5</v>
@@ -4224,16 +4191,16 @@
         <v>44.5</v>
       </c>
       <c r="D128" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F128" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="G128" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H128" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="I128" t="s">
         <v>5</v>
@@ -4250,16 +4217,16 @@
         <v>43.8</v>
       </c>
       <c r="D129" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F129" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="G129" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H129" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="I129" t="s">
         <v>5</v>
@@ -4276,16 +4243,16 @@
         <v>45</v>
       </c>
       <c r="D130" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F130" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="G130" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H130" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="I130" t="s">
         <v>5</v>
@@ -4302,16 +4269,16 @@
         <v>44.5</v>
       </c>
       <c r="D131" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F131" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="G131" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H131" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="I131" t="s">
         <v>5</v>
@@ -4328,16 +4295,16 @@
         <v>43.8</v>
       </c>
       <c r="D132" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F132" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="G132" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H132" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="I132" t="s">
         <v>5</v>
@@ -4354,16 +4321,16 @@
         <v>42</v>
       </c>
       <c r="D133" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F133" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="G133" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H133" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="I133" t="s">
         <v>5</v>
@@ -4380,16 +4347,16 @@
         <v>42</v>
       </c>
       <c r="D134" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F134" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="G134" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H134" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="I134" t="s">
         <v>5</v>
@@ -4406,16 +4373,16 @@
         <v>42</v>
       </c>
       <c r="D135" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F135" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="G135" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H135" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="I135" t="s">
         <v>5</v>
@@ -4432,16 +4399,16 @@
         <v>42</v>
       </c>
       <c r="D136" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F136" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="G136" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H136" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="I136" t="s">
         <v>5</v>
@@ -4458,16 +4425,16 @@
         <v>42.5</v>
       </c>
       <c r="D137" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F137" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="G137" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H137" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="I137" t="s">
         <v>5</v>
@@ -4484,16 +4451,16 @@
         <v>42</v>
       </c>
       <c r="D138" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F138" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="G138" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H138" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="I138" t="s">
         <v>5</v>
@@ -4510,16 +4477,16 @@
         <v>43</v>
       </c>
       <c r="D139" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F139" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="G139" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H139" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="I139" t="s">
         <v>5</v>
@@ -4536,16 +4503,16 @@
         <v>42</v>
       </c>
       <c r="D140" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F140" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="G140" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H140" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="I140" t="s">
         <v>5</v>
@@ -4562,16 +4529,16 @@
         <v>39.5</v>
       </c>
       <c r="D141" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F141" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="G141" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H141" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="I141" t="s">
         <v>5</v>
@@ -4588,16 +4555,16 @@
         <v>39.5</v>
       </c>
       <c r="D142" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F142" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="G142" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H142" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="I142" t="s">
         <v>5</v>
@@ -4614,16 +4581,16 @@
         <v>39.5</v>
       </c>
       <c r="D143" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F143" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="G143" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H143" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="I143" t="s">
         <v>5</v>
@@ -4640,19 +4607,19 @@
         <v>38.4</v>
       </c>
       <c r="D144" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E144" t="s">
         <v>18</v>
       </c>
       <c r="F144" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="G144" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H144" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="I144" t="s">
         <v>5</v>
@@ -4669,16 +4636,16 @@
         <v>40.5</v>
       </c>
       <c r="D145" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F145" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="G145" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H145" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="I145" t="s">
         <v>5</v>
@@ -4695,16 +4662,16 @@
         <v>40</v>
       </c>
       <c r="D146" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F146" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="G146" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H146" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="I146" t="s">
         <v>5</v>
@@ -4721,16 +4688,16 @@
         <v>40.200000000000003</v>
       </c>
       <c r="D147" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F147" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="G147" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H147" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="I147" t="s">
         <v>5</v>
@@ -4747,16 +4714,16 @@
         <v>39.6</v>
       </c>
       <c r="D148" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F148" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="G148" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H148" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="I148" t="s">
         <v>5</v>
@@ -4773,16 +4740,16 @@
         <v>39.5</v>
       </c>
       <c r="D149" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F149" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="G149" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H149" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="I149" t="s">
         <v>5</v>
@@ -4799,16 +4766,16 @@
         <v>39.700000000000003</v>
       </c>
       <c r="D150" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F150" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="G150" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H150" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="I150" t="s">
         <v>5</v>
@@ -4825,16 +4792,16 @@
         <v>39.799999999999997</v>
       </c>
       <c r="D151" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F151" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="G151" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H151" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="I151" t="s">
         <v>5</v>
@@ -4848,22 +4815,22 @@
         <v>39.5</v>
       </c>
       <c r="C152">
-        <v>38.1</v>
+        <v>36.700000000000003</v>
       </c>
       <c r="D152" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E152" t="s">
         <v>12</v>
       </c>
       <c r="F152" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="G152" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H152" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I152" t="s">
         <v>5</v>
@@ -4877,22 +4844,22 @@
         <v>39.5</v>
       </c>
       <c r="C153">
-        <v>38.1</v>
+        <v>36.5</v>
       </c>
       <c r="D153" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E153" t="s">
         <v>12</v>
       </c>
       <c r="F153" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="G153" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H153" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I153" t="s">
         <v>5</v>
@@ -4906,22 +4873,22 @@
         <v>39.799999999999997</v>
       </c>
       <c r="C154">
-        <v>38.1</v>
+        <v>37.4</v>
       </c>
       <c r="D154" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E154" t="s">
         <v>18</v>
       </c>
       <c r="F154" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="G154" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H154" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I154" t="s">
         <v>5</v>
@@ -4938,19 +4905,19 @@
         <v>38.1</v>
       </c>
       <c r="D155" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E155" t="s">
         <v>19</v>
       </c>
       <c r="F155" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="G155" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H155" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I155" t="s">
         <v>5</v>
@@ -4967,19 +4934,19 @@
         <v>38.1</v>
       </c>
       <c r="D156" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E156" t="s">
         <v>19</v>
       </c>
       <c r="F156" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="G156" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H156" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I156" t="s">
         <v>5</v>
@@ -4996,19 +4963,19 @@
         <v>38.1</v>
       </c>
       <c r="D157" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E157" t="s">
         <v>19</v>
       </c>
       <c r="F157" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="G157" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H157" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I157" t="s">
         <v>5</v>
@@ -5025,19 +4992,19 @@
         <v>38.1</v>
       </c>
       <c r="D158" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E158" t="s">
         <v>19</v>
       </c>
       <c r="F158" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="G158" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H158" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I158" t="s">
         <v>5</v>
@@ -5054,19 +5021,19 @@
         <v>38.1</v>
       </c>
       <c r="D159" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E159" t="s">
         <v>19</v>
       </c>
       <c r="F159" s="1" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="G159" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H159" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I159" t="s">
         <v>5</v>
@@ -5083,19 +5050,19 @@
         <v>38.1</v>
       </c>
       <c r="D160" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E160" t="s">
         <v>19</v>
       </c>
       <c r="F160" s="1" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="G160" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H160" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I160" t="s">
         <v>5</v>
@@ -5112,19 +5079,19 @@
         <v>37.200000000000003</v>
       </c>
       <c r="D161" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E161" t="s">
         <v>18</v>
       </c>
       <c r="F161" s="1" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="G161" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H161" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I161" t="s">
         <v>5</v>
@@ -5141,19 +5108,19 @@
         <v>37.700000000000003</v>
       </c>
       <c r="D162" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E162" t="s">
         <v>19</v>
       </c>
       <c r="F162" s="1" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="G162" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H162" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I162" t="s">
         <v>5</v>
@@ -5170,19 +5137,19 @@
         <v>38.1</v>
       </c>
       <c r="D163" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E163" t="s">
         <v>19</v>
       </c>
       <c r="F163" s="1" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="G163" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H163" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I163" t="s">
         <v>5</v>
@@ -5199,19 +5166,19 @@
         <v>38.200000000000003</v>
       </c>
       <c r="D164" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E164" t="s">
         <v>19</v>
       </c>
       <c r="F164" s="1" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="G164" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H164" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I164" t="s">
         <v>5</v>
@@ -5228,19 +5195,19 @@
         <v>37.799999999999997</v>
       </c>
       <c r="D165" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E165" t="s">
         <v>18</v>
       </c>
       <c r="F165" s="1" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="G165" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H165" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I165" t="s">
         <v>5</v>
@@ -5257,19 +5224,19 @@
         <v>38.299999999999997</v>
       </c>
       <c r="D166" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E166" t="s">
         <v>19</v>
       </c>
       <c r="F166" s="1" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="G166" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H166" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I166" t="s">
         <v>5</v>
@@ -5286,16 +5253,16 @@
         <v>38.1</v>
       </c>
       <c r="D167" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F167" s="1" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="G167" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H167" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I167" t="s">
         <v>5</v>
@@ -5312,19 +5279,19 @@
         <v>37.700000000000003</v>
       </c>
       <c r="D168" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E168" t="s">
         <v>19</v>
       </c>
       <c r="F168" s="1" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="G168" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H168" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I168" t="s">
         <v>5</v>
@@ -5341,19 +5308,19 @@
         <v>37.799999999999997</v>
       </c>
       <c r="D169" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E169" t="s">
         <v>19</v>
       </c>
       <c r="F169" s="1" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="G169" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H169" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I169" t="s">
         <v>5</v>
@@ -5370,16 +5337,16 @@
         <v>36</v>
       </c>
       <c r="D170" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F170" s="1" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="G170" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H170" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I170" t="s">
         <v>5</v>
@@ -5396,16 +5363,16 @@
         <v>36.200000000000003</v>
       </c>
       <c r="D171" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F171" s="1" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="G171" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H171" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I171" t="s">
         <v>5</v>
@@ -5422,16 +5389,16 @@
         <v>36.5</v>
       </c>
       <c r="D172" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F172" s="1" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="G172" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H172" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I172" t="s">
         <v>5</v>
@@ -5448,16 +5415,16 @@
         <v>39.200000000000003</v>
       </c>
       <c r="D173" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F173" s="1" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="G173" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H173" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I173" t="s">
         <v>5</v>
@@ -5474,19 +5441,19 @@
         <v>38.1</v>
       </c>
       <c r="D174" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E174" t="s">
         <v>19</v>
       </c>
       <c r="F174" s="1" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="G174" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H174" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I174" t="s">
         <v>5</v>
@@ -5503,16 +5470,16 @@
         <v>38.299999999999997</v>
       </c>
       <c r="D175" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F175" s="1" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="G175" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H175" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I175" t="s">
         <v>5</v>
@@ -5529,19 +5496,19 @@
         <v>38</v>
       </c>
       <c r="D176" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E176" t="s">
         <v>19</v>
       </c>
       <c r="F176" s="1" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="G176" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H176" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I176" t="s">
         <v>5</v>
@@ -5558,16 +5525,16 @@
         <v>38.200000000000003</v>
       </c>
       <c r="D177" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F177" s="1" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="G177" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H177" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I177" t="s">
         <v>5</v>
@@ -5584,19 +5551,19 @@
         <v>38</v>
       </c>
       <c r="D178" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E178" t="s">
         <v>12</v>
       </c>
       <c r="F178" s="1" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G178" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H178" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="I178" t="s">
         <v>5</v>
@@ -5613,19 +5580,19 @@
         <v>36</v>
       </c>
       <c r="D179" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F179" s="1" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="G179" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H179" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="I179" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
     </row>
     <row r="180" spans="1:9">
@@ -5639,19 +5606,19 @@
         <v>36</v>
       </c>
       <c r="D180" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F180" s="1" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="G180" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H180" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="I180" t="s">
-        <v>48</v>
+        <v>5</v>
       </c>
     </row>
     <row r="181" spans="1:9">
@@ -5665,19 +5632,19 @@
         <v>36</v>
       </c>
       <c r="D181" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F181" s="1" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="G181" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H181" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="I181" t="s">
-        <v>49</v>
+        <v>5</v>
       </c>
     </row>
     <row r="182" spans="1:9">
@@ -5691,19 +5658,19 @@
         <v>36</v>
       </c>
       <c r="D182" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F182" s="1" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="G182" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H182" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="I182" t="s">
-        <v>50</v>
+        <v>5</v>
       </c>
     </row>
     <row r="183" spans="1:9">
@@ -5717,19 +5684,19 @@
         <v>36</v>
       </c>
       <c r="D183" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F183" s="1" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="G183" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H183" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="I183" t="s">
-        <v>51</v>
+        <v>5</v>
       </c>
     </row>
     <row r="184" spans="1:9">
@@ -5743,19 +5710,19 @@
         <v>36</v>
       </c>
       <c r="D184" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F184" s="1" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="G184" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H184" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="I184" t="s">
-        <v>53</v>
+        <v>5</v>
       </c>
     </row>
     <row r="185" spans="1:9">
@@ -5769,22 +5736,22 @@
         <v>33</v>
       </c>
       <c r="D185" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E185" t="s">
         <v>18</v>
       </c>
       <c r="F185" s="1" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="G185" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H185" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="I185" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
     </row>
     <row r="186" spans="1:9">
@@ -5798,19 +5765,19 @@
         <v>35</v>
       </c>
       <c r="D186" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F186" s="1" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="G186" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H186" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="I186" t="s">
-        <v>55</v>
+        <v>5</v>
       </c>
     </row>
     <row r="187" spans="1:9">
@@ -5824,22 +5791,22 @@
         <v>33.6</v>
       </c>
       <c r="D187" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E187" t="s">
         <v>18</v>
       </c>
       <c r="F187" s="1" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="G187" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H187" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="I187" t="s">
-        <v>56</v>
+        <v>5</v>
       </c>
     </row>
     <row r="188" spans="1:9">
@@ -5853,19 +5820,19 @@
         <v>33.1</v>
       </c>
       <c r="D188" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F188" s="1" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="G188" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H188" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="I188" t="s">
-        <v>57</v>
+        <v>5</v>
       </c>
     </row>
     <row r="189" spans="1:9">
@@ -5879,19 +5846,19 @@
         <v>35.6</v>
       </c>
       <c r="D189" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="F189" s="1" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="G189" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H189" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="I189" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
     </row>
     <row r="190" spans="1:9">
@@ -5905,19 +5872,19 @@
         <v>83.5</v>
       </c>
       <c r="D190" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="F190" s="2" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="G190" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="H190" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="I190" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
     </row>
     <row r="191" spans="1:9">
@@ -5931,19 +5898,19 @@
         <v>76</v>
       </c>
       <c r="D191" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="F191" s="2" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="G191" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="H191" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="I191" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
     </row>
     <row r="192" spans="1:9">
@@ -5957,19 +5924,19 @@
         <v>91.1</v>
       </c>
       <c r="D192" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="F192" s="2" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="G192" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="H192" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="I192" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
     </row>
     <row r="193" spans="1:9">
@@ -5983,19 +5950,19 @@
         <v>79.7</v>
       </c>
       <c r="D193" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="F193" s="2" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="G193" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="H193" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="I193" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
     </row>
     <row r="194" spans="1:9">
@@ -6009,19 +5976,19 @@
         <v>77.3</v>
       </c>
       <c r="D194" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="F194" s="2" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="G194" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="H194" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="I194" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
     </row>
     <row r="195" spans="1:9">
@@ -6035,19 +6002,19 @@
         <v>87.5</v>
       </c>
       <c r="D195" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="F195" s="2" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="G195" t="s">
+        <v>112</v>
+      </c>
+      <c r="H195" t="s">
         <v>123</v>
       </c>
-      <c r="H195" t="s">
-        <v>134</v>
-      </c>
       <c r="I195" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
     </row>
     <row r="196" spans="1:9">
@@ -6061,19 +6028,19 @@
         <v>95.5</v>
       </c>
       <c r="D196" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="F196" s="2" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="G196" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="H196" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="I196" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
     </row>
     <row r="197" spans="1:9">
@@ -6087,19 +6054,19 @@
         <v>85.9</v>
       </c>
       <c r="D197" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="F197" s="2" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="G197" t="s">
+        <v>112</v>
+      </c>
+      <c r="H197" t="s">
         <v>123</v>
       </c>
-      <c r="H197" t="s">
-        <v>134</v>
-      </c>
       <c r="I197" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
     </row>
     <row r="198" spans="1:9">
@@ -6113,17 +6080,17 @@
         <v>86.1</v>
       </c>
       <c r="D198" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="F198" s="2"/>
       <c r="G198" t="s">
+        <v>112</v>
+      </c>
+      <c r="H198" t="s">
         <v>123</v>
       </c>
-      <c r="H198" t="s">
-        <v>134</v>
-      </c>
       <c r="I198" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
     </row>
     <row r="199" spans="1:9">
@@ -6137,16 +6104,16 @@
         <v>87.5</v>
       </c>
       <c r="D199" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="G199" t="s">
+        <v>112</v>
+      </c>
+      <c r="H199" t="s">
         <v>123</v>
       </c>
-      <c r="H199" t="s">
-        <v>134</v>
-      </c>
       <c r="I199" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
     </row>
     <row r="200" spans="1:9">
@@ -6162,19 +6129,19 @@
         <v>-39.104548110000003</v>
       </c>
       <c r="D200" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="F200" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="G200" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="H200" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="I200" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
     </row>
     <row r="201" spans="1:9">
@@ -6190,19 +6157,19 @@
         <v>-38.531135749999997</v>
       </c>
       <c r="D201" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="F201" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="G201" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="H201" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="I201" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
     </row>
     <row r="202" spans="1:9">
@@ -6218,19 +6185,19 @@
         <v>-38.6166883</v>
       </c>
       <c r="D202" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="F202" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="G202" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="H202" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="I202" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
     </row>
     <row r="203" spans="1:9">
@@ -6246,19 +6213,19 @@
         <v>-38.369071699999999</v>
       </c>
       <c r="D203" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="F203" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="G203" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="H203" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="I203" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
     </row>
     <row r="204" spans="1:9">
@@ -6273,19 +6240,19 @@
         <v>-39.104548110000003</v>
       </c>
       <c r="D204" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="F204" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="G204" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="H204" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="I204" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
     </row>
     <row r="205" spans="1:9">
@@ -6300,19 +6267,19 @@
         <v>-39.48480979</v>
       </c>
       <c r="D205" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="F205" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="G205" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="H205" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="I205" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
     </row>
     <row r="206" spans="1:9">
@@ -6327,19 +6294,19 @@
         <v>-38.369071699999999</v>
       </c>
       <c r="D206" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="F206" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="G206" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="H206" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="I206" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
     </row>
     <row r="207" spans="1:9">
@@ -6354,19 +6321,19 @@
         <v>-39.104548110000003</v>
       </c>
       <c r="D207" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="F207" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="G207" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="H207" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="I207" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
     </row>
     <row r="208" spans="1:9">
@@ -6381,19 +6348,19 @@
         <v>-38.369071699999999</v>
       </c>
       <c r="D208" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="F208" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="G208" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="H208" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="I208" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
     </row>
     <row r="209" spans="1:9">
@@ -6408,19 +6375,19 @@
         <v>-41.243539550000001</v>
       </c>
       <c r="D209" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="F209" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="G209" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="H209" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="I209" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>